<commit_message>
📊 Actualización automática del dashboard
</commit_message>
<xml_diff>
--- a/Comentarios Campaña.xlsx
+++ b/Comentarios Campaña.xlsx
@@ -8,10 +8,6 @@
   </bookViews>
   <sheets>
     <sheet name="Comentarios" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Resumen_Posts" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Stats_Plataforma" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="URLs_Fallidas" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Stats_Extraccion" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -6056,1750 +6052,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G45"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>post_number</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>platform</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>post_url</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Total_Comentarios</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Total_Likes</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Primera_Extraccion</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Ultima_Extraccion</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Facebook</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/100064867445065/posts/pfbid02wii1P1pD2H7gkGwQfcYVVDWuGRYjto2YEykU9x3EViVfR74LZVBZjDGKtTGUNs5l</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Facebook</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/100064867445065/posts/pfbid0KW1D1SQ7N3wkb6y3CghuTp8cCTqL7spikmcNds9w8dXUWbZoqf4PGtW1TCFC4mBdl</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Facebook</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/100064867445065/posts/pfbid0HdzfymKuNH5WHHiBr2w9GheCM5tjxp9SDPbiWX83wFUVFAQbj1A5fzaiB5BgrP34l</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Facebook</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/100064867445065/posts/pfbid0jqKsZHCWqyFzLmcCQ1DVBQKxhACNHVh8NrXTvpiWeBjuEwYAumJXpougMVRoKX31l</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Facebook</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/100064867445065/posts/pfbid06rYqXZEpGhYe2vcmZ5WfevUVLR1AhYePytnJmqt6kk525bMTpDjhDwoJpgpkyWrWl</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Facebook</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/reel/3261599530668110/</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Facebook</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/share/p/1EVoU9fDD6/</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>0</v>
-      </c>
-      <c r="E8" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Facebook</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/share/v/18vjmR9EbP/</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
-        <v>0</v>
-      </c>
-      <c r="E9" t="n">
-        <v>0</v>
-      </c>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Facebook</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/share/p/19G6LM1Pof/</t>
-        </is>
-      </c>
-      <c r="D10" t="n">
-        <v>0</v>
-      </c>
-      <c r="E10" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Facebook</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/share/v/1JB8tmKYtm/</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" t="n">
-        <v>0</v>
-      </c>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" t="n">
-        <v>11</v>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Instagram</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/p/DZNxPDAALy4/</t>
-        </is>
-      </c>
-      <c r="D12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E12" t="n">
-        <v>0</v>
-      </c>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" t="n">
-        <v>12</v>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Instagram</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/p/DZNxHkkgASI/</t>
-        </is>
-      </c>
-      <c r="D13" t="n">
-        <v>0</v>
-      </c>
-      <c r="E13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" t="n">
-        <v>13</v>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Instagram</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/p/DZMS8j3gLwc/</t>
-        </is>
-      </c>
-      <c r="D14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" t="n">
-        <v>14</v>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Instagram</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/p/DZMSywUgClm/</t>
-        </is>
-      </c>
-      <c r="D15" t="n">
-        <v>0</v>
-      </c>
-      <c r="E15" t="n">
-        <v>0</v>
-      </c>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" t="n">
-        <v>15</v>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Instagram</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/p/DZLkuhcgMiD/</t>
-        </is>
-      </c>
-      <c r="D16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E16" t="n">
-        <v>0</v>
-      </c>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" t="n">
-        <v>16</v>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Instagram</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/p/DZgJjAmgNkB/</t>
-        </is>
-      </c>
-      <c r="D17" t="n">
-        <v>0</v>
-      </c>
-      <c r="E17" t="n">
-        <v>0</v>
-      </c>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" t="n">
-        <v>17</v>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Instagram</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/p/DZ5ypteA0CO/</t>
-        </is>
-      </c>
-      <c r="D18" t="n">
-        <v>0</v>
-      </c>
-      <c r="E18" t="n">
-        <v>0</v>
-      </c>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" t="n">
-        <v>18</v>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Instagram</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/p/DZ5t8kSAvF3/</t>
-        </is>
-      </c>
-      <c r="D19" t="n">
-        <v>0</v>
-      </c>
-      <c r="E19" t="n">
-        <v>0</v>
-      </c>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" t="n">
-        <v>19</v>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Instagram</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/p/DZ5yxYgAy5c/</t>
-        </is>
-      </c>
-      <c r="D20" t="n">
-        <v>2</v>
-      </c>
-      <c r="E20" t="n">
-        <v>0</v>
-      </c>
-      <c r="F20" s="1" t="n">
-        <v>46210.59957175926</v>
-      </c>
-      <c r="G20" s="1" t="n">
-        <v>46211.58980324074</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="n">
-        <v>20</v>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Instagram</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/p/DZ5zHVwAbLS/</t>
-        </is>
-      </c>
-      <c r="D21" t="n">
-        <v>0</v>
-      </c>
-      <c r="E21" t="n">
-        <v>0</v>
-      </c>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" t="n">
-        <v>21</v>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Facebook</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/100064867445065/posts/pfbid02awSRn7qMHiopGBURJWVj5Yqv6Kxy5dgs7RKPfdZSLYSd2ZUZkJv52cwE582X2XyFl</t>
-        </is>
-      </c>
-      <c r="D22" t="n">
-        <v>12</v>
-      </c>
-      <c r="E22" t="n">
-        <v>1</v>
-      </c>
-      <c r="F22" s="1" t="n">
-        <v>46220.97578703704</v>
-      </c>
-      <c r="G22" s="1" t="n">
-        <v>46259.67501157407</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="n">
-        <v>22</v>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Facebook</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/100064867445065/posts/pfbid0diXSKWcBuTriKjD7Nwt6JVvYPUCCtYhUPBXacCtRb66LmEM7VnPzk5mNx4SPFu81l</t>
-        </is>
-      </c>
-      <c r="D23" t="n">
-        <v>14</v>
-      </c>
-      <c r="E23" t="n">
-        <v>1</v>
-      </c>
-      <c r="F23" s="1" t="n">
-        <v>46217.89942129629</v>
-      </c>
-      <c r="G23" s="1" t="n">
-        <v>46243.94265046297</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="n">
-        <v>23</v>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Facebook</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/100064867445065/posts/pfbid0u3H29b1191LidQ6R4ScnVbymeypHNjdJZgFg9d7fSGNsjJzHXvKF8W1yBTzet227l</t>
-        </is>
-      </c>
-      <c r="D24" t="n">
-        <v>0</v>
-      </c>
-      <c r="E24" t="n">
-        <v>0</v>
-      </c>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" t="n">
-        <v>24</v>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Facebook</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/100064867445065/posts/pfbid02RJW4as6otnHmCuYRMm2c5Uh2KDJvcJykcUsjmRwGtE3BEJobZjT8PosVhhqKGQvYl</t>
-        </is>
-      </c>
-      <c r="D25" t="n">
-        <v>0</v>
-      </c>
-      <c r="E25" t="n">
-        <v>0</v>
-      </c>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" t="n">
-        <v>25</v>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Facebook</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/100064867445065/posts/pfbid02jvvAfrhCFmzTnxK1pvNmh15Y8qThsqiWPocQ9dUo3kETV4HhCXc3ZffrAaq4gEHrl</t>
-        </is>
-      </c>
-      <c r="D26" t="n">
-        <v>11</v>
-      </c>
-      <c r="E26" t="n">
-        <v>3</v>
-      </c>
-      <c r="F26" s="1" t="n">
-        <v>46221.04325231481</v>
-      </c>
-      <c r="G26" s="1" t="n">
-        <v>46255.09995370371</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="n">
-        <v>26</v>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Facebook</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/100064867445065/posts/pfbid02c5QGzXhE2N8V1K1dYhrycRLWmoqMyPgLhkoUWws3WrATKMY3QeVVcgeSE9mTM73Ll</t>
-        </is>
-      </c>
-      <c r="D27" t="n">
-        <v>8</v>
-      </c>
-      <c r="E27" t="n">
-        <v>0</v>
-      </c>
-      <c r="F27" s="1" t="n">
-        <v>46219.06762731481</v>
-      </c>
-      <c r="G27" s="1" t="n">
-        <v>46257.370625</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="n">
-        <v>27</v>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Facebook</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/100064867445065/posts/pfbid0ZQYTeNNy2eTtEqRUWUG3sno85TQAQEpp1UC65toR11BoHe3VFGVtckUw4Sf7bAVFl</t>
-        </is>
-      </c>
-      <c r="D28" t="n">
-        <v>0</v>
-      </c>
-      <c r="E28" t="n">
-        <v>0</v>
-      </c>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" t="n">
-        <v>28</v>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Facebook</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/100064867445065/posts/pfbid02MxKsxXBXFoAXeZcMJQ3Qn8BrrisRTgMzVgtbyNssSZf4nLr47uJCMFKPzs8wWYGhl</t>
-        </is>
-      </c>
-      <c r="D29" t="n">
-        <v>0</v>
-      </c>
-      <c r="E29" t="n">
-        <v>0</v>
-      </c>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" t="n">
-        <v>29</v>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Facebook</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/100064867445065/posts/pfbid0jxSvw9oJXMG8A9eNrYVsqbDjjpFB4wAe6hpkFkKpK5TzU6AHetEfBbNHp7m6gHLil</t>
-        </is>
-      </c>
-      <c r="D30" t="n">
-        <v>6</v>
-      </c>
-      <c r="E30" t="n">
-        <v>2</v>
-      </c>
-      <c r="F30" s="1" t="n">
-        <v>46232.85341435186</v>
-      </c>
-      <c r="G30" s="1" t="n">
-        <v>46257.19048611111</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="n">
-        <v>30</v>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>Facebook</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/100064867445065/posts/pfbid029TVtHR1KfaW4AsBqfonhJ1VHSfG32B4BmVrYEXwaXxRBm6npftXSEnoxPPs5zpEYl</t>
-        </is>
-      </c>
-      <c r="D31" t="n">
-        <v>4</v>
-      </c>
-      <c r="E31" t="n">
-        <v>0</v>
-      </c>
-      <c r="F31" s="1" t="n">
-        <v>46226.95178240741</v>
-      </c>
-      <c r="G31" s="1" t="n">
-        <v>46247.0819212963</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="n">
-        <v>31</v>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>Facebook</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/100064867445065/posts/pfbid0LSCGwRefL4RtjMGDw8x4sPBjcpUvG5Nb7sspUQA3u2FxNKfKPce62zJbG84DLiNrl</t>
-        </is>
-      </c>
-      <c r="D32" t="n">
-        <v>0</v>
-      </c>
-      <c r="E32" t="n">
-        <v>0</v>
-      </c>
-      <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" t="n">
-        <v>32</v>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Facebook</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/100064867445065/posts/pfbid06cvKsDX83RU1JegqcrpMTftA37dFcZNmD3rHssE245K5AzJfVim7LbydRbMvPedgl</t>
-        </is>
-      </c>
-      <c r="D33" t="n">
-        <v>0</v>
-      </c>
-      <c r="E33" t="n">
-        <v>0</v>
-      </c>
-      <c r="F33" t="inlineStr"/>
-      <c r="G33" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="A34" t="n">
-        <v>33</v>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Instagram</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/p/Dao8BvHgwPO/</t>
-        </is>
-      </c>
-      <c r="D34" t="n">
-        <v>0</v>
-      </c>
-      <c r="E34" t="n">
-        <v>0</v>
-      </c>
-      <c r="F34" t="inlineStr"/>
-      <c r="G34" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" t="n">
-        <v>34</v>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Instagram</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/p/Dax0GBqgVfJ/</t>
-        </is>
-      </c>
-      <c r="D35" t="n">
-        <v>2</v>
-      </c>
-      <c r="E35" t="n">
-        <v>2</v>
-      </c>
-      <c r="F35" s="1" t="n">
-        <v>46240.25452546297</v>
-      </c>
-      <c r="G35" s="1" t="n">
-        <v>46253.70673611111</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="n">
-        <v>35</v>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>Instagram</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/p/Dao9WjmA7W6/</t>
-        </is>
-      </c>
-      <c r="D36" t="n">
-        <v>0</v>
-      </c>
-      <c r="E36" t="n">
-        <v>0</v>
-      </c>
-      <c r="F36" t="inlineStr"/>
-      <c r="G36" t="inlineStr"/>
-    </row>
-    <row r="37">
-      <c r="A37" t="n">
-        <v>36</v>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>Instagram</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/p/DaxwTQ4gyKQ/</t>
-        </is>
-      </c>
-      <c r="D37" t="n">
-        <v>0</v>
-      </c>
-      <c r="E37" t="n">
-        <v>0</v>
-      </c>
-      <c r="F37" t="inlineStr"/>
-      <c r="G37" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="A38" t="n">
-        <v>37</v>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>Instagram</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/p/Dao_lUkAI8z/</t>
-        </is>
-      </c>
-      <c r="D38" t="n">
-        <v>0</v>
-      </c>
-      <c r="E38" t="n">
-        <v>0</v>
-      </c>
-      <c r="F38" t="inlineStr"/>
-      <c r="G38" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="A39" t="n">
-        <v>38</v>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>Instagram</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/p/DaxyhZDAdzK/</t>
-        </is>
-      </c>
-      <c r="D39" t="n">
-        <v>1</v>
-      </c>
-      <c r="E39" t="n">
-        <v>0</v>
-      </c>
-      <c r="F39" s="1" t="n">
-        <v>46259.18921296296</v>
-      </c>
-      <c r="G39" s="1" t="n">
-        <v>46259.18921296296</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="n">
-        <v>39</v>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>Instagram</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/p/DapAo_QgLPK/</t>
-        </is>
-      </c>
-      <c r="D40" t="n">
-        <v>0</v>
-      </c>
-      <c r="E40" t="n">
-        <v>0</v>
-      </c>
-      <c r="F40" t="inlineStr"/>
-      <c r="G40" t="inlineStr"/>
-    </row>
-    <row r="41">
-      <c r="A41" t="n">
-        <v>40</v>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>Instagram</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/p/DaxzJ8jgGVl/</t>
-        </is>
-      </c>
-      <c r="D41" t="n">
-        <v>0</v>
-      </c>
-      <c r="E41" t="n">
-        <v>0</v>
-      </c>
-      <c r="F41" t="inlineStr"/>
-      <c r="G41" t="inlineStr"/>
-    </row>
-    <row r="42">
-      <c r="A42" t="n">
-        <v>41</v>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>Instagram</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/p/Dao-Ke_AEaE/</t>
-        </is>
-      </c>
-      <c r="D42" t="n">
-        <v>0</v>
-      </c>
-      <c r="E42" t="n">
-        <v>0</v>
-      </c>
-      <c r="F42" t="inlineStr"/>
-      <c r="G42" t="inlineStr"/>
-    </row>
-    <row r="43">
-      <c r="A43" t="n">
-        <v>42</v>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>Instagram</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/p/Dax0ftQgN6m/</t>
-        </is>
-      </c>
-      <c r="D43" t="n">
-        <v>1</v>
-      </c>
-      <c r="E43" t="n">
-        <v>0</v>
-      </c>
-      <c r="F43" s="1" t="n">
-        <v>46229.43672453704</v>
-      </c>
-      <c r="G43" s="1" t="n">
-        <v>46229.43672453704</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="n">
-        <v>43</v>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>Instagram</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/p/Dao_BRHA1YQ/</t>
-        </is>
-      </c>
-      <c r="D44" t="n">
-        <v>0</v>
-      </c>
-      <c r="E44" t="n">
-        <v>0</v>
-      </c>
-      <c r="F44" t="inlineStr"/>
-      <c r="G44" t="inlineStr"/>
-    </row>
-    <row r="45">
-      <c r="A45" t="n">
-        <v>44</v>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>Instagram</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/p/Daxx_DygJuZ/</t>
-        </is>
-      </c>
-      <c r="D45" t="n">
-        <v>0</v>
-      </c>
-      <c r="E45" t="n">
-        <v>0</v>
-      </c>
-      <c r="F45" t="inlineStr"/>
-      <c r="G45" t="inlineStr"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>platform</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Total_Posts</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Total_Comentarios</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Promedio_Likes</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Total_Likes</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Facebook</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>6</v>
-      </c>
-      <c r="C2" t="n">
-        <v>55</v>
-      </c>
-      <c r="D2" t="n">
-        <v>0.13</v>
-      </c>
-      <c r="E2" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Instagram</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>4</v>
-      </c>
-      <c r="C3" t="n">
-        <v>6</v>
-      </c>
-      <c r="D3" t="n">
-        <v>0.33</v>
-      </c>
-      <c r="E3" t="n">
-        <v>2</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B41"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>URL</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/100064867445065/posts/pfbid02wii1P1pD2H7gkGwQfcYVVDWuGRYjto2YEykU9x3EViVfR74LZVBZjDGKtTGUNs5l</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>FAILED_ALL_ATTEMPTS</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/100064867445065/posts/pfbid0KW1D1SQ7N3wkb6y3CghuTp8cCTqL7spikmcNds9w8dXUWbZoqf4PGtW1TCFC4mBdl</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>FAILED_ALL_ATTEMPTS</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/100064867445065/posts/pfbid0HdzfymKuNH5WHHiBr2w9GheCM5tjxp9SDPbiWX83wFUVFAQbj1A5fzaiB5BgrP34l</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>FAILED_ALL_ATTEMPTS</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/100064867445065/posts/pfbid0jqKsZHCWqyFzLmcCQ1DVBQKxhACNHVh8NrXTvpiWeBjuEwYAumJXpougMVRoKX31l</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>FAILED_ALL_ATTEMPTS</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/100064867445065/posts/pfbid06rYqXZEpGhYe2vcmZ5WfevUVLR1AhYePytnJmqt6kk525bMTpDjhDwoJpgpkyWrWl</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>FAILED_ALL_ATTEMPTS</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/reel/3261599530668110/</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>FAILED_ALL_ATTEMPTS</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/share/p/1EVoU9fDD6/</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>FAILED_ALL_ATTEMPTS</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/share/v/18vjmR9EbP/</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>FAILED_ALL_ATTEMPTS</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/share/p/19G6LM1Pof/</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>FAILED_ALL_ATTEMPTS</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/share/v/1JB8tmKYtm/</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>FAILED_ALL_ATTEMPTS</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/100064867445065/posts/pfbid02awSRn7qMHiopGBURJWVj5Yqv6Kxy5dgs7RKPfdZSLYSd2ZUZkJv52cwE582X2XyFl</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>FAILED_ALL_ATTEMPTS</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/100064867445065/posts/pfbid0diXSKWcBuTriKjD7Nwt6JVvYPUCCtYhUPBXacCtRb66LmEM7VnPzk5mNx4SPFu81l</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>FAILED_ALL_ATTEMPTS</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/100064867445065/posts/pfbid0u3H29b1191LidQ6R4ScnVbymeypHNjdJZgFg9d7fSGNsjJzHXvKF8W1yBTzet227l</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>FAILED_ALL_ATTEMPTS</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/100064867445065/posts/pfbid02RJW4as6otnHmCuYRMm2c5Uh2KDJvcJykcUsjmRwGtE3BEJobZjT8PosVhhqKGQvYl</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>FAILED_ALL_ATTEMPTS</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/100064867445065/posts/pfbid02jvvAfrhCFmzTnxK1pvNmh15Y8qThsqiWPocQ9dUo3kETV4HhCXc3ZffrAaq4gEHrl</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>FAILED_ALL_ATTEMPTS</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/100064867445065/posts/pfbid02c5QGzXhE2N8V1K1dYhrycRLWmoqMyPgLhkoUWws3WrATKMY3QeVVcgeSE9mTM73Ll</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>FAILED_ALL_ATTEMPTS</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/100064867445065/posts/pfbid0ZQYTeNNy2eTtEqRUWUG3sno85TQAQEpp1UC65toR11BoHe3VFGVtckUw4Sf7bAVFl</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>FAILED_ALL_ATTEMPTS</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/100064867445065/posts/pfbid02MxKsxXBXFoAXeZcMJQ3Qn8BrrisRTgMzVgtbyNssSZf4nLr47uJCMFKPzs8wWYGhl</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>FAILED_ALL_ATTEMPTS</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/100064867445065/posts/pfbid0jxSvw9oJXMG8A9eNrYVsqbDjjpFB4wAe6hpkFkKpK5TzU6AHetEfBbNHp7m6gHLil</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>FAILED_ALL_ATTEMPTS</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/100064867445065/posts/pfbid029TVtHR1KfaW4AsBqfonhJ1VHSfG32B4BmVrYEXwaXxRBm6npftXSEnoxPPs5zpEYl</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>FAILED_ALL_ATTEMPTS</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/100064867445065/posts/pfbid0LSCGwRefL4RtjMGDw8x4sPBjcpUvG5Nb7sspUQA3u2FxNKfKPce62zJbG84DLiNrl</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>FAILED_ALL_ATTEMPTS</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/100064867445065/posts/pfbid06cvKsDX83RU1JegqcrpMTftA37dFcZNmD3rHssE245K5AzJfVim7LbydRbMvPedgl</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>FAILED_ALL_ATTEMPTS</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/p/DZNxPDAALy4/</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>FAILED_ALL_ATTEMPTS</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/p/DZNxHkkgASI/</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>FAILED_ALL_ATTEMPTS</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/p/DZMS8j3gLwc/</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>FAILED_ALL_ATTEMPTS</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/p/DZMSywUgClm/</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>FAILED_ALL_ATTEMPTS</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/p/DZLkuhcgMiD/</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>FAILED_ALL_ATTEMPTS</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/p/DZgJjAmgNkB/</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>FAILED_ALL_ATTEMPTS</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/p/DZ5ypteA0CO/</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>FAILED_ALL_ATTEMPTS</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/p/DZ5t8kSAvF3/</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>FAILED_ALL_ATTEMPTS</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/p/DZ5zHVwAbLS/</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>FAILED_ALL_ATTEMPTS</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/p/Dao8BvHgwPO/</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>FAILED_ALL_ATTEMPTS</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/p/Dao9WjmA7W6/</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>FAILED_ALL_ATTEMPTS</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/p/DaxwTQ4gyKQ/</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>FAILED_ALL_ATTEMPTS</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/p/Dao_lUkAI8z/</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>FAILED_ALL_ATTEMPTS</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/p/DapAo_QgLPK/</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>FAILED_ALL_ATTEMPTS</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/p/DaxzJ8jgGVl/</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>FAILED_ALL_ATTEMPTS</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/p/Dao-Ke_AEaE/</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>FAILED_ALL_ATTEMPTS</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/p/Dao_BRHA1YQ/</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>FAILED_ALL_ATTEMPTS</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/p/Daxx_DygJuZ/</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>FAILED_ALL_ATTEMPTS</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>total_attempts</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>successful</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>failed</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>no_comments</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>invalid_comments</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
-        <v>44</v>
-      </c>
-      <c r="B2" t="n">
-        <v>4</v>
-      </c>
-      <c r="C2" t="n">
-        <v>40</v>
-      </c>
-      <c r="D2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E2" t="n">
-        <v>124</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>